<commit_message>
re-run meme70, TFM report draft functionally complete
</commit_message>
<xml_diff>
--- a/Supplementary Material/Precision-Recall-F1 Calculator.xlsx
+++ b/Supplementary Material/Precision-Recall-F1 Calculator.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enoch/Documents/Local Erill Research/drippy/Supplementary Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93054235-E65B-844C-92BC-3032247BB606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F477A89D-F3B3-2E4F-A96E-BCB5823002CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14700" yWindow="760" windowWidth="14700" windowHeight="18360" xr2:uid="{29BA5AF6-D670-8442-A245-123F22FD2C81}"/>
+    <workbookView xWindow="14700" yWindow="760" windowWidth="14700" windowHeight="18360" activeTab="1" xr2:uid="{29BA5AF6-D670-8442-A245-123F22FD2C81}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="40_CollecTF" sheetId="1" r:id="rId1"/>
+    <sheet name="70_MEME" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="9">
   <si>
     <t>Precision</t>
   </si>
@@ -174,13 +175,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -196,6 +197,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>241300</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{158979E6-6D23-41F7-9669-B8479EBE97FD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="2819400"/>
+          <a:ext cx="6997700" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -529,7 +579,7 @@
       <c r="C1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
     </row>
@@ -537,18 +587,18 @@
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="6">
         <f xml:space="preserve"> F2/(F2+F4)</f>
         <v>0.90909090909090906</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="6">
         <f>F8/(F8+F10)</f>
         <v>0.967741935483871</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="5">
         <v>20</v>
       </c>
     </row>
@@ -556,18 +606,18 @@
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="6">
         <f xml:space="preserve"> F2 / (F2+F5)</f>
         <v>0.76923076923076927</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="6">
         <f>F8/(F8+F11)</f>
         <v>0.69767441860465118</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="5">
         <v>41</v>
       </c>
     </row>
@@ -575,68 +625,197 @@
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="6">
         <f>2*(B2*B3) / (B2+B3)</f>
         <v>0.83333333333333326</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="6">
         <f>2*(C2*C3) / (C2+C3)</f>
         <v>0.81081081081081097</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="5"/>
-      <c r="E5" s="6" t="s">
+      <c r="A5" s="4"/>
+      <c r="E5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="5"/>
+      <c r="A6" s="4"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="5">
         <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="5">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="5">
         <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4985F019-34FC-CC4C-B91A-F46A0B97EA45}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="6">
+        <f xml:space="preserve"> F2/(F2+F4)</f>
+        <v>1</v>
+      </c>
+      <c r="C2" s="6">
+        <f>F8/(F8+F10)</f>
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6">
+        <f xml:space="preserve"> F2 / (F2+F5)</f>
+        <v>0.6</v>
+      </c>
+      <c r="C3" s="6">
+        <f>F8/(F8+F11)</f>
+        <v>1</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="5">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="6">
+        <f>2*(B2*B3) / (B2+B3)</f>
+        <v>0.74999999999999989</v>
+      </c>
+      <c r="C4" s="6">
+        <f>2*(C2*C3) / (C2+C3)</f>
+        <v>0.88</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="4"/>
+      <c r="E5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E7" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E8" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" s="5">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="5">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="5">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>